<commit_message>
data: publish 2026-09-22 sampler-linked operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-09-22-182路.xlsx
+++ b/data/export/2026-09-22-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC10"/>
+  <dimension ref="A1:AC17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -637,24 +637,24 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>07:10</t>
+          <t>07:16</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>66分钟</t>
+          <t>71分钟</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>06:21采样：该车到重点站德川路华夏东路 ETA 2分钟；叠加该车自身同类时段从该站到终点历史中位数47分钟，约±5分钟</t>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -693,12 +693,12 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>同车重点站剩余时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr">
@@ -708,22 +708,22 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA2" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>79.0</t>
         </is>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>1/9</t>
+          <t>5/13</t>
         </is>
       </c>
     </row>
@@ -756,24 +756,24 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>07:18</t>
+          <t>07:23</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>69分钟</t>
+          <t>73分钟</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>06:21采样：该车到重点站博兴路东陆路 ETA 2分钟；叠加该车自身同类时段从该站到终点历史中位数55分钟，约±5分钟</t>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -812,12 +812,12 @@
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>同车重点站剩余时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr">
@@ -837,12 +837,12 @@
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>73.0</t>
         </is>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>2/9</t>
+          <t>2/13</t>
         </is>
       </c>
     </row>
@@ -875,29 +875,29 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>70分钟</t>
+          <t>71分钟</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>06:21采样：该车到重点站德川路华夏东路 ETA 18分钟；叠加该车自身同类时段从该站到终点历史中位数50分钟，约±5分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -931,12 +931,12 @@
       </c>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>同车重点站剩余时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr">
@@ -946,22 +946,22 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>78.5</t>
         </is>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>3/9</t>
+          <t>4/13</t>
         </is>
       </c>
     </row>
@@ -994,29 +994,29 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>07:53</t>
+          <t>07:58</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>78分钟</t>
+          <t>83分钟</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数78分钟估算，约±5分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1050,12 +1050,12 @@
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y5" s="2" t="inlineStr">
@@ -1075,12 +1075,12 @@
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
-          <t>78.0</t>
+          <t>83.0</t>
         </is>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>5/9</t>
+          <t>8/13</t>
         </is>
       </c>
     </row>
@@ -1118,26 +1118,22 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>08:06</t>
+          <t>08:02</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>91分钟</t>
+          <t>88分钟</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数91分钟估算，约±12分钟</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
+          <t>SHMAAS末次终点ETA推算：07:21采样，终点ETA 41分钟</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -1145,7 +1141,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1174,7 +1170,7 @@
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>末次终点ETA兜底</t>
         </is>
       </c>
       <c r="Y6" s="2" t="inlineStr">
@@ -1184,22 +1180,22 @@
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
-          <t>91.0</t>
+          <t>83.5</t>
         </is>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>8/9</t>
+          <t>9/13</t>
         </is>
       </c>
     </row>
@@ -1249,12 +1245,12 @@
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数72分钟估算，约±8分钟</t>
+          <t>07:21采样：该车到重点站唐陆公路唐镇路 ETA 0分钟；叠加该车自身同类时段从该站到终点历史中位数38分钟，约±6分钟</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1264,7 +1260,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1293,7 +1289,7 @@
       </c>
       <c r="X7" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>同车重点站剩余时间</t>
         </is>
       </c>
       <c r="Y7" s="2" t="inlineStr">
@@ -1318,7 +1314,7 @@
       </c>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>4/9</t>
+          <t>1/13</t>
         </is>
       </c>
     </row>
@@ -1356,22 +1352,26 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>08:26</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>92分钟</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr"/>
+          <t>07:21采样：该车到重点站唐陆公路创新路 ETA 37分钟；叠加该车自身同类时段从该站到终点历史中位数28分钟，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -1379,7 +1379,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1403,17 +1403,17 @@
       </c>
       <c r="W8" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X8" s="2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>同车重点站剩余时间</t>
         </is>
       </c>
       <c r="Y8" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z8" s="2" t="inlineStr">
@@ -1423,13 +1423,17 @@
       </c>
       <c r="AA8" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB8" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB8" s="2" t="inlineStr">
+        <is>
+          <t>92.0</t>
+        </is>
+      </c>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>13/13</t>
         </is>
       </c>
     </row>
@@ -1467,24 +1471,24 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>08:25</t>
+          <t>08:17</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>85分钟</t>
+          <t>78分钟</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数85分钟估算，约±8分钟</t>
+          <t>07:21采样：该车到重点站唐陆公路唐镇路 ETA 6分钟；叠加该车自身同类时段从该站到终点历史中位数50分钟，约±11分钟</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1494,7 +1498,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1518,12 +1522,12 @@
       </c>
       <c r="W9" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>同车重点站剩余时间</t>
         </is>
       </c>
       <c r="Y9" s="2" t="inlineStr">
@@ -1543,12 +1547,12 @@
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
-          <t>85.0</t>
+          <t>78.0</t>
         </is>
       </c>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>6/9</t>
+          <t>3/13</t>
         </is>
       </c>
     </row>
@@ -1556,24 +1560,24 @@
       <c r="A10" s="2" t="inlineStr"/>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>沪A32298D</t>
+          <t>沪A35717D</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
           <t>金杨路金口路</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>07:15</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>川沙客运站</t>
-        </is>
-      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -1586,34 +1590,34 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>08:42</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>87分钟</t>
+          <t>79分钟</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数87分钟估算，约±8分钟</t>
+          <t>07:21采样：该车到重点站新德西路德翔路 ETA 14分钟；叠加该车自身同类时段从该站到终点历史中位数55分钟，约±5分钟</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>06:02</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1627,47 +1631,880 @@
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr">
         <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>同车重点站剩余时间</t>
+        </is>
+      </c>
+      <c r="Y10" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB10" s="2" t="inlineStr">
+        <is>
+          <t>79.0</t>
+        </is>
+      </c>
+      <c r="AC10" s="2" t="inlineStr">
+        <is>
+          <t>5/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>沪A32298D</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
           <t>07:15</t>
         </is>
       </c>
-      <c r="V10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>08:43</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>89分钟</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>07:21采样：该车到重点站东陆路金海路 ETA 22分钟；叠加该车自身同类时段从该站到终点历史中位数60分钟，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
         <is>
           <t>计划发车</t>
         </is>
       </c>
-      <c r="W10" s="2" t="inlineStr">
+      <c r="W11" s="2" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="X10" s="2" t="inlineStr">
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>同车重点站剩余时间</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr">
+        <is>
+          <t>89.0</t>
+        </is>
+      </c>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>11/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>沪A31073D</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>08:51</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>87分钟</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数87分钟估算，约±6分钟</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
         <is>
           <t>同车历史全程时间</t>
         </is>
       </c>
-      <c r="Y10" s="2" t="inlineStr">
+      <c r="Y12" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="Z10" s="2" t="inlineStr">
+      <c r="Z12" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA10" s="2" t="inlineStr">
+      <c r="AA12" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AB10" s="2" t="inlineStr">
+      <c r="AB12" s="2" t="inlineStr">
         <is>
           <t>87.0</t>
         </is>
       </c>
-      <c r="AC10" s="2" t="inlineStr">
-        <is>
-          <t>7/9</t>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>10/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>沪A68397D</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>09:02</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>87分钟</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数87分钟估算，约±9分钟</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB13" s="2" t="inlineStr">
+        <is>
+          <t>79.0</t>
+        </is>
+      </c>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>5/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>沪A55712D</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>08:57</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>82分钟</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数82分钟估算，约±14分钟</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>07:11</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr">
+        <is>
+          <t>82.0</t>
+        </is>
+      </c>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>7/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>沪A12050A</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>09:18</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>90分钟</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数90分钟估算，约±12分钟</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr">
+        <is>
+          <t>90.0</t>
+        </is>
+      </c>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>12/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>沪A68870D</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>09:21</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>86分钟</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数86分钟估算，约±6分钟</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y16" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA16" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB16" s="2" t="inlineStr">
+        <is>
+          <t>78.5</t>
+        </is>
+      </c>
+      <c r="AC16" s="2" t="inlineStr">
+        <is>
+          <t>4/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>79分钟</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数79分钟估算，约±9分钟</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB17" s="2" t="inlineStr">
+        <is>
+          <t>83.5</t>
+        </is>
+      </c>
+      <c r="AC17" s="2" t="inlineStr">
+        <is>
+          <t>9/13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: publish 2026-09-22 rolling operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-09-22-182路.xlsx
+++ b/data/export/2026-09-22-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC25"/>
+  <dimension ref="A1:AC27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -669,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -708,22 +708,22 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA2" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
-          <t>85.5</t>
+          <t>84.0</t>
         </is>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>5/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>3/14</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>1/14</t>
+          <t>2/14</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1075,12 +1075,12 @@
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
-          <t>87.5</t>
+          <t>84.5</t>
         </is>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>8/14</t>
+          <t>7/14</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1313,12 +1313,12 @@
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
-          <t>85.5</t>
+          <t>84.5</t>
         </is>
       </c>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>5/14</t>
+          <t>7/14</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1502,7 +1502,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>2/14</t>
+          <t>3/14</t>
         </is>
       </c>
     </row>
@@ -1594,24 +1594,24 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>08:43</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>91分钟</t>
+          <t>92分钟</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+          <t>SHMAAS终点近站ETA直接确认，约±2分钟</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1670,12 +1670,12 @@
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>90.5</t>
         </is>
       </c>
       <c r="AC10" s="2" t="inlineStr">
         <is>
-          <t>9/14</t>
+          <t>11/14</t>
         </is>
       </c>
     </row>
@@ -1713,24 +1713,24 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>08:49</t>
+          <t>08:48</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>94分钟</t>
+          <t>93分钟</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1789,12 +1789,12 @@
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>89.5</t>
         </is>
       </c>
       <c r="AC11" s="2" t="inlineStr">
         <is>
-          <t>9/14</t>
+          <t>10/14</t>
         </is>
       </c>
     </row>
@@ -1827,7 +1827,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1837,17 +1837,21 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>97分钟</t>
+          <t>96分钟</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>SHMAAS末次终点ETA推算：08:22采样，终点ETA 38分钟</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -1855,7 +1859,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1879,12 +1883,12 @@
       </c>
       <c r="W12" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X12" s="2" t="inlineStr">
         <is>
-          <t>末次终点ETA兜底</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y12" s="2" t="inlineStr">
@@ -1894,22 +1898,22 @@
       </c>
       <c r="Z12" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA12" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
-          <t>97.0</t>
+          <t>87.5</t>
         </is>
       </c>
       <c r="AC12" s="2" t="inlineStr">
         <is>
-          <t>14/14</t>
+          <t>9/14</t>
         </is>
       </c>
     </row>
@@ -1942,12 +1946,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>09:14</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1959,12 +1963,12 @@
       <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>08:22采样：该车到重点站唐陆公路川桥路 ETA 0分钟；叠加该车自身同类时段从该站到终点历史中位数52分钟，约±5分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -1974,7 +1978,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1998,12 +2002,12 @@
       </c>
       <c r="W13" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X13" s="2" t="inlineStr">
         <is>
-          <t>同车重点站剩余时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y13" s="2" t="inlineStr">
@@ -2013,22 +2017,22 @@
       </c>
       <c r="Z13" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA13" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
-          <t>85.5</t>
+          <t>84.0</t>
         </is>
       </c>
       <c r="AC13" s="2" t="inlineStr">
         <is>
-          <t>5/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -2066,24 +2070,24 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>90分钟</t>
+          <t>100分钟</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>08:22采样：该车到重点站唐陆公路川桥路 ETA 14分钟；叠加该车自身同类时段从该站到终点历史中位数29分钟，约±6分钟</t>
+          <t>08:43采样：该车到重点站佳林路金高路 ETA 10分钟；叠加该车自身同类时段从该站到终点历史中位数22分钟，约±5分钟</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -2093,7 +2097,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -2142,12 +2146,12 @@
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="AC14" s="2" t="inlineStr">
         <is>
-          <t>9/14</t>
+          <t>14/14</t>
         </is>
       </c>
     </row>
@@ -2185,24 +2189,24 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>09:22</t>
+          <t>09:23</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>94分钟</t>
+          <t>96分钟</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>08:12采样：该车到重点站新德西路德川路 ETA 1分钟；叠加该车自身同类时段从该站到终点历史中位数68分钟，约±6分钟</t>
+          <t>08:43采样：该车到重点站唐陆公路锦绣东路 ETA 3分钟；叠加该车自身同类时段从该站到终点历史中位数37分钟，约±5分钟</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -2212,7 +2216,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>08:12</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -2261,7 +2265,7 @@
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
-          <t>94.0</t>
+          <t>96.0</t>
         </is>
       </c>
       <c r="AC15" s="2" t="inlineStr">
@@ -2304,7 +2308,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>09:25</t>
+          <t>09:26</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -2316,12 +2320,12 @@
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>08:22采样：该车到重点站唐陆公路川桥路 ETA 11分钟；叠加该车自身同类时段从该站到终点历史中位数52分钟，约±5分钟</t>
+          <t>08:43采样：该车到重点站唐陆公路春雅路 ETA 4分钟；叠加该车自身同类时段从该站到终点历史中位数39分钟，约±7分钟</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -2331,7 +2335,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -2385,7 +2389,7 @@
       </c>
       <c r="AC16" s="2" t="inlineStr">
         <is>
-          <t>1/14</t>
+          <t>2/14</t>
         </is>
       </c>
     </row>
@@ -2423,7 +2427,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>09:32</t>
+          <t>09:31</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -2435,12 +2439,12 @@
       <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>08:22采样：该车到重点站德川路华夏东路 ETA 6分钟；叠加该车自身同类时段从该站到终点历史中位数63分钟，约±7分钟</t>
+          <t>08:43采样：该车到重点站唐陆公路锦绣东路 ETA 10分钟；叠加该车自身同类时段从该站到终点历史中位数38分钟，约±5分钟</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -2450,7 +2454,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -2504,7 +2508,7 @@
       </c>
       <c r="AC17" s="2" t="inlineStr">
         <is>
-          <t>3/14</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -2542,19 +2546,19 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>09:48</t>
+          <t>09:43</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>94分钟</t>
+          <t>88分钟</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>08:22采样：该车到重点站新川路华东路 ETA 10分钟；叠加该车自身同类时段从该站到终点历史中位数76分钟，约±5分钟</t>
+          <t>08:43采样：该车到重点站唐陆公路唐镇路 ETA 6分钟；叠加该车自身同类时段从该站到终点历史中位数54分钟，约±5分钟</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -2569,7 +2573,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -2618,12 +2622,12 @@
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
-          <t>87.5</t>
+          <t>84.5</t>
         </is>
       </c>
       <c r="AC18" s="2" t="inlineStr">
         <is>
-          <t>8/14</t>
+          <t>7/14</t>
         </is>
       </c>
     </row>
@@ -2661,7 +2665,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>09:37</t>
+          <t>09:36</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -2673,12 +2677,12 @@
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>08:22采样：该车到重点站博兴路东陆路 ETA 11分钟；叠加该车自身同类时段从该站到终点历史中位数63分钟，约±11分钟</t>
+          <t>08:43采样：该车到重点站唐陆公路春雅路 ETA 15分钟；叠加该车自身同类时段从该站到终点历史中位数38分钟，约±5分钟</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
@@ -2688,7 +2692,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -2712,7 +2716,7 @@
       </c>
       <c r="W19" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="X19" s="2" t="inlineStr">
@@ -2742,7 +2746,7 @@
       </c>
       <c r="AC19" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -2780,19 +2784,19 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>09:57</t>
+          <t>09:52</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>86分钟</t>
+          <t>81分钟</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数86分钟估算，约±14分钟</t>
+          <t>08:43采样：该车到重点站唐陆公路唐镇路 ETA 21分钟；叠加该车自身同类时段从该站到终点历史中位数48分钟，约±14分钟</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
@@ -2807,7 +2811,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2836,7 +2840,7 @@
       </c>
       <c r="X20" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>同车重点站剩余时间</t>
         </is>
       </c>
       <c r="Y20" s="2" t="inlineStr">
@@ -2856,12 +2860,12 @@
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
-          <t>86.0</t>
+          <t>81.0</t>
         </is>
       </c>
       <c r="AC20" s="2" t="inlineStr">
         <is>
-          <t>7/14</t>
+          <t>1/14</t>
         </is>
       </c>
     </row>
@@ -2899,19 +2903,19 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>10:03</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>88分钟</t>
+          <t>86分钟</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数88分钟估算，约±8分钟</t>
+          <t>08:43采样：该车到重点站东陆路金海路 ETA 18分钟；叠加该车自身同类时段从该站到终点历史中位数60分钟，约±8分钟</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -2926,7 +2930,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2955,7 +2959,7 @@
       </c>
       <c r="X21" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>同车重点站剩余时间</t>
         </is>
       </c>
       <c r="Y21" s="2" t="inlineStr">
@@ -2975,12 +2979,12 @@
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
-          <t>85.5</t>
+          <t>84.5</t>
         </is>
       </c>
       <c r="AC21" s="2" t="inlineStr">
         <is>
-          <t>5/14</t>
+          <t>7/14</t>
         </is>
       </c>
     </row>
@@ -3045,7 +3049,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -3164,7 +3168,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
@@ -3218,7 +3222,7 @@
       </c>
       <c r="AC23" s="2" t="inlineStr">
         <is>
-          <t>2/14</t>
+          <t>3/14</t>
         </is>
       </c>
     </row>
@@ -3283,7 +3287,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -3332,12 +3336,12 @@
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>89.5</t>
         </is>
       </c>
       <c r="AC24" s="2" t="inlineStr">
         <is>
-          <t>9/14</t>
+          <t>10/14</t>
         </is>
       </c>
     </row>
@@ -3402,7 +3406,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -3451,12 +3455,250 @@
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>90.5</t>
         </is>
       </c>
       <c r="AC25" s="2" t="inlineStr">
         <is>
+          <t>11/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr"/>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>沪A31073D</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>09:22</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>10:41</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>79分钟</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数79分钟估算，约±8分钟</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>08:43</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="inlineStr"/>
+      <c r="S26" s="2" t="inlineStr"/>
+      <c r="T26" s="2" t="inlineStr"/>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
+          <t>09:22</t>
+        </is>
+      </c>
+      <c r="V26" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W26" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X26" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y26" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z26" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA26" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB26" s="2" t="inlineStr">
+        <is>
+          <t>87.5</t>
+        </is>
+      </c>
+      <c r="AC26" s="2" t="inlineStr">
+        <is>
           <t>9/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr"/>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>沪A68397D</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>81分钟</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数81分钟估算，约±8分钟</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>08:43</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q27" s="2" t="inlineStr"/>
+      <c r="R27" s="2" t="inlineStr"/>
+      <c r="S27" s="2" t="inlineStr"/>
+      <c r="T27" s="2" t="inlineStr"/>
+      <c r="U27" s="2" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="V27" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W27" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X27" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y27" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z27" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA27" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB27" s="2" t="inlineStr">
+        <is>
+          <t>84.0</t>
+        </is>
+      </c>
+      <c r="AC27" s="2" t="inlineStr">
+        <is>
+          <t>6/14</t>
         </is>
       </c>
     </row>

</xml_diff>